<commit_message>
docs: reword workbook README sheets
</commit_message>
<xml_diff>
--- a/inputs/execution/firm_capacity_fallbacks_by_cr.xlsx
+++ b/inputs/execution/firm_capacity_fallbacks_by_cr.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luisfernando\Desktop\OSeMOSYS\OSTRAM_storage_debug_try2\t1_confection\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luisfernando\Desktop\OSeMOSYS\OSTRAM_main\inputs\execution\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46BCE03C-D416-4F11-A2FA-BF8702EA5404}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E0104D2-4174-4F00-9494-F235236F21D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-76920" yWindow="-4080" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-4080" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="fallbacks" sheetId="1" r:id="rId1"/>
@@ -65,9 +65,6 @@
     <t>Purpose</t>
   </si>
   <si>
-    <t>Per-country-region fallback values for the careful XLSX reserve-margin patcher.</t>
-  </si>
-  <si>
     <t>Stock cap</t>
   </si>
   <si>
@@ -83,9 +80,6 @@
     <t>Sentinel behavior</t>
   </si>
   <si>
-    <t>The patcher only replaces existing cap values equal to 0 or 9999 by default.</t>
-  </si>
-  <si>
     <t>Starting assumption</t>
   </si>
   <si>
@@ -96,6 +90,12 @@
   </si>
   <si>
     <t>TECH_PREFIX and YEAR can be added to the fallbacks sheet for more specific overrides.</t>
+  </si>
+  <si>
+    <t>The adjustment only replaces existing cap values equal to 0 or 9999 by default.</t>
+  </si>
+  <si>
+    <t>Per-country-region fallback values for the careful XLSX reserve-margin adjustment.</t>
   </si>
 </sst>
 </file>
@@ -601,47 +601,47 @@
         <v>13</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
         <v>15</v>
-      </c>
-      <c r="B2" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
         <v>17</v>
-      </c>
-      <c r="B3" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>